<commit_message>
Update Zenodo links to v2 (23491480), remove obsolete weights draft, and clean reading list
</commit_message>
<xml_diff>
--- a/data/literature/Apiary_Literature_Reading_List.xlsx
+++ b/data/literature/Apiary_Literature_Reading_List.xlsx
@@ -607,7 +607,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Expert-knowledge hierarchical fuzzy inference system (13 variables/43 rules simplified to 5/6). Criteria: temperature, humidity, wind, precipitation, solar radiation, land use (crop types), slope, aspect, distance to water, distance to transport. No numeric weights. Possibly related to the Ecol. Informatics expert-knowledge paper (pii S1574954124000724) but that pii was NOT seen/confirmed.</t>
+          <t>Expert-knowledge hierarchical fuzzy inference system (13 variables/43 rules simplified to 5/6). Criteria: temperature, humidity, wind, precipitation, solar radiation, land use (crop types), slope, aspect, distance to water, distance to transport. No numeric weights.</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr"/>
@@ -624,13 +624,13 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Abou-Shaara, H.F. (per caller; author not displayed on page)</t>
+          <t>Abou-Shaara, H.F.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>GIS Analysis to Locate More Suitable Wintering Areas for Honey [Bees...] (title truncated in URL)</t>
+          <t>GIS Analysis to Locate More Suitable Wintering Areas for Honey Bees</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -655,7 +655,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>GIS suitability of wintering areas for honey bees. Page bot-blocked; criteria/weights not verified.</t>
+          <t>GIS suitability of wintering areas for honey bees. Criteria/weights not verified.</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr"/>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>GIS-MCE with stakeholder/expert participation, La Union, Philippines. Criteria/weights not on page. Page shows chapter DOI 10.1007/978-94-007-0671-2_13 (book version); caller's RJAS DOI 10.3923/rjasci.2010.242.253 not seen.</t>
+          <t>GIS-MCE with stakeholder/expert participation, La Union, Philippines. Criteria/weights not on page. Related chapter DOI 10.1007/978-94-007-0671-2_13; RJAS DOI 10.3923/rjasci.2010.242.253.</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr"/>
@@ -2003,7 +2003,7 @@
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>Compares MCDA techniques (AHP, TOPSIS, VIKOR per Rojas-Briceño 2026 review). Criteria: slope, elevation, aspect, precipitation, flora, distance to water, roads, settlements. Weights not on repository page. Caller-supplied DOI 10.1007/s13592-020-00736-7 not seen in this session.</t>
+          <t>Compares MCDA techniques (AHP, TOPSIS, VIKOR per Rojas-Briceño 2026 review). Criteria: slope, elevation, aspect, precipitation, flora, distance to water, roads, settlements. Weights not on repository page (DOI: 10.1007/s13592-020-00736-7).</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr"/>

</xml_diff>